<commit_message>
ll searching ai, empty lines
</commit_message>
<xml_diff>
--- a/LL/excel_sablon.xlsx
+++ b/LL/excel_sablon.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zsomborgalgoczi/Desktop/label labor assets/label_generator_excels/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zsomborgalgoczi/Desktop/workspace/github.com/zsombzs/label_generator/LL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03AD74F0-11B9-6E43-8216-D88F8EF629CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D205B0E-8B80-ED4A-8F34-E5D94DC40DD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" xr2:uid="{195B7CB8-57D0-714D-A057-F87136F4FC09}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Cikkszám</t>
   </si>
@@ -51,6 +51,24 @@
   </si>
   <si>
     <t>Ár</t>
+  </si>
+  <si>
+    <t>8711347001576</t>
+  </si>
+  <si>
+    <t>8711347000012</t>
+  </si>
+  <si>
+    <t>8711347000050</t>
+  </si>
+  <si>
+    <t>8711347000067</t>
+  </si>
+  <si>
+    <t>8711347000111</t>
+  </si>
+  <si>
+    <t>8711347000135</t>
   </si>
 </sst>
 </file>
@@ -169,14 +187,14 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -511,14 +529,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0807640-E514-5C42-8365-97613778117F}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="35.1640625" style="7" customWidth="1"/>
+    <col min="1" max="1" width="35.1640625" style="5" customWidth="1"/>
     <col min="2" max="2" width="29.33203125" customWidth="1"/>
     <col min="3" max="3" width="33.33203125" customWidth="1"/>
     <col min="4" max="4" width="27.33203125" customWidth="1"/>
-    <col min="5" max="5" width="29" style="5" customWidth="1"/>
+    <col min="5" max="5" width="29" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="43" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -539,8 +557,52 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="6"/>
-      <c r="B2" s="4"/>
+      <c r="A2" s="6">
+        <v>100001</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="6">
+        <v>100002</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="6">
+        <v>100003</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="6">
+        <v>100004</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="6">
+        <v>100005</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="6">
+        <v>100006</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
new sale label prototype, drop
</commit_message>
<xml_diff>
--- a/LL/excel_sablon.xlsx
+++ b/LL/excel_sablon.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zsomborgalgoczi/Desktop/workspace/github.com/zsombzs/label_generator/LL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D205B0E-8B80-ED4A-8F34-E5D94DC40DD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F21618EB-CA35-7842-8CDB-38A88DA10233}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" xr2:uid="{195B7CB8-57D0-714D-A057-F87136F4FC09}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Cikkszám</t>
   </si>
@@ -69,6 +69,9 @@
   </si>
   <si>
     <t>8711347000135</t>
+  </si>
+  <si>
+    <t>Akciós_ár</t>
   </si>
 </sst>
 </file>
@@ -529,17 +532,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0807640-E514-5C42-8365-97613778117F}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.1640625" style="5" customWidth="1"/>
     <col min="2" max="2" width="29.33203125" customWidth="1"/>
     <col min="3" max="3" width="33.33203125" customWidth="1"/>
     <col min="4" max="4" width="27.33203125" customWidth="1"/>
-    <col min="5" max="5" width="29" style="4" customWidth="1"/>
+    <col min="5" max="6" width="29" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="43" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="43" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -555,8 +558,11 @@
       <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A2" s="6">
         <v>100001</v>
       </c>
@@ -564,7 +570,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="6">
         <v>100002</v>
       </c>
@@ -572,7 +578,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="6">
         <v>100003</v>
       </c>
@@ -580,7 +586,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="6">
         <v>100004</v>
       </c>
@@ -588,7 +594,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="6">
         <v>100005</v>
       </c>
@@ -596,7 +602,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="6">
         <v>100006</v>
       </c>

</xml_diff>

<commit_message>
ritzer, ll for the video
</commit_message>
<xml_diff>
--- a/LL/excel_sablon.xlsx
+++ b/LL/excel_sablon.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zsomborgalgoczi/Desktop/workspace/github.com/zsombzs/label_generator/LL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F21618EB-CA35-7842-8CDB-38A88DA10233}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA7FB13A-1B3D-F344-97AA-2DC0CA14D2E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" xr2:uid="{195B7CB8-57D0-714D-A057-F87136F4FC09}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>Cikkszám</t>
   </si>
@@ -51,27 +51,6 @@
   </si>
   <si>
     <t>Ár</t>
-  </si>
-  <si>
-    <t>8711347001576</t>
-  </si>
-  <si>
-    <t>8711347000012</t>
-  </si>
-  <si>
-    <t>8711347000050</t>
-  </si>
-  <si>
-    <t>8711347000067</t>
-  </si>
-  <si>
-    <t>8711347000111</t>
-  </si>
-  <si>
-    <t>8711347000135</t>
-  </si>
-  <si>
-    <t>Akciós_ár</t>
   </si>
 </sst>
 </file>
@@ -532,17 +511,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0807640-E514-5C42-8365-97613778117F}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.1640625" style="5" customWidth="1"/>
     <col min="2" max="2" width="29.33203125" customWidth="1"/>
     <col min="3" max="3" width="33.33203125" customWidth="1"/>
     <col min="4" max="4" width="27.33203125" customWidth="1"/>
-    <col min="5" max="6" width="29" style="4" customWidth="1"/>
+    <col min="5" max="5" width="29" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="43" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="43" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -558,57 +537,30 @@
       <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="6">
-        <v>100001</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="6">
-        <v>100002</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="6">
-        <v>100003</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="6">
-        <v>100004</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="6">
-        <v>100005</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="6">
-        <v>100006</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>10</v>
-      </c>
+    </row>
+    <row r="2" spans="1:5" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="6"/>
+      <c r="B2" s="7"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="6"/>
+      <c r="B3" s="7"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="6"/>
+      <c r="B4" s="7"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="6"/>
+      <c r="B5" s="7"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="6"/>
+      <c r="B6" s="7"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="6"/>
+      <c r="B7" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>